<commit_message>
fix algorithm for label positioning
</commit_message>
<xml_diff>
--- a/files/results_cut.xlsx
+++ b/files/results_cut.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="846" activeTab="6"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="846" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="23">
   <si>
     <t>Title</t>
   </si>
@@ -244,7 +244,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -259,6 +259,10 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -282,10 +286,7 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -597,18 +598,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="10"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -785,27 +786,27 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:K12"/>
+  <dimension ref="B2:U22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="11" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="6" t="s">
+    <row r="2" spans="2:21" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
-    </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="10"/>
+    </row>
+    <row r="3" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -817,7 +818,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
     </row>
-    <row r="4" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2"/>
       <c r="C4" s="1" t="s">
         <v>1</v>
@@ -847,260 +848,833 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1">
         <v>1</v>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="6">
         <v>0.1240967364599086</v>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="6">
         <v>0.33120990323358379</v>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="6">
         <v>5.4772255750516613E-2</v>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="6">
         <v>0.20099751242241781</v>
       </c>
-      <c r="G5" s="15">
+      <c r="G5" s="6">
         <v>0.34438350715445132</v>
       </c>
-      <c r="H5" s="15">
+      <c r="H5" s="6">
         <v>0.30364452901377947</v>
       </c>
-      <c r="I5" s="15">
+      <c r="I5" s="6">
         <v>0.41892720131306832</v>
       </c>
-      <c r="J5" s="15">
+      <c r="J5" s="6">
         <v>0.1187434208703792</v>
       </c>
-      <c r="K5" s="15">
+      <c r="K5" s="6">
         <v>0.40323690307311899</v>
       </c>
     </row>
-    <row r="6" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <v>2</v>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="6">
         <v>7.0710678118654766E-2</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="6">
         <v>6.4807406984078608E-2</v>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="6">
         <v>0.198997487421324</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="6">
         <v>0.1048808848170152</v>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="6">
         <v>5.0990195135927847E-2</v>
       </c>
-      <c r="H6" s="15">
+      <c r="H6" s="6">
         <v>0.18055470085267791</v>
       </c>
-      <c r="I6" s="15">
+      <c r="I6" s="6">
         <v>8.5440037453175313E-2</v>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="6">
         <v>4.123105625617661E-2</v>
       </c>
-      <c r="K6" s="15">
+      <c r="K6" s="6">
         <v>0.62233431530006444</v>
       </c>
     </row>
-    <row r="7" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="1">
         <v>3</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="6">
         <v>0.16309506430300089</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="6">
         <v>0.43023249528597912</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="6">
         <v>9.8488578017961043E-2</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="6">
         <v>0.21563858652847831</v>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="6">
         <v>0.42118879377305368</v>
       </c>
-      <c r="H7" s="15">
+      <c r="H7" s="6">
         <v>0.1367479433117734</v>
       </c>
-      <c r="I7" s="15">
+      <c r="I7" s="6">
         <v>0.35693136595149488</v>
       </c>
-      <c r="J7" s="15">
+      <c r="J7" s="6">
         <v>9.9498743710662002E-2</v>
       </c>
-      <c r="K7" s="15">
+      <c r="K7" s="6">
         <v>0.39522145690739008</v>
       </c>
     </row>
-    <row r="8" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="1">
         <v>4</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="6">
         <v>0.1889444362769119</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="6">
         <v>0.21470910553583891</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="6">
         <v>0.1374772708486752</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="6">
         <v>0.1523154621172782</v>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="6">
         <v>0.1772004514666935</v>
       </c>
-      <c r="H8" s="15">
+      <c r="H8" s="6">
         <v>0.34539832078341087</v>
       </c>
-      <c r="I8" s="15">
+      <c r="I8" s="6">
         <v>0.28390139133156778</v>
       </c>
-      <c r="J8" s="15">
+      <c r="J8" s="6">
         <v>8.6023252670426265E-2</v>
       </c>
-      <c r="K8" s="15">
+      <c r="K8" s="6">
         <v>1.094714574672321</v>
       </c>
     </row>
-    <row r="9" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="1">
         <v>5</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="6">
         <v>0.1212435565298214</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="6">
         <v>0.24919871588754219</v>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="6">
         <v>9.6436507609929556E-2</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="6">
         <v>0.18138357147217049</v>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="6">
         <v>0.2861817604250837</v>
       </c>
-      <c r="H9" s="15">
+      <c r="H9" s="6">
         <v>0.18165902124584951</v>
       </c>
-      <c r="I9" s="15">
+      <c r="I9" s="6">
         <v>0.48249352327259282</v>
       </c>
-      <c r="J9" s="15">
+      <c r="J9" s="6">
         <v>8.306623862918075E-2</v>
       </c>
-      <c r="K9" s="15">
+      <c r="K9" s="6">
         <v>2.178577517555893</v>
       </c>
     </row>
-    <row r="10" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1">
         <v>6</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="6">
         <v>0.41448763552125412</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="6">
         <v>9.0553851381374159E-2</v>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="6">
         <v>0.10049875621120891</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="6">
         <v>0.2929163703175362</v>
       </c>
-      <c r="G10" s="15">
+      <c r="G10" s="6">
         <v>0.1118033988749895</v>
       </c>
-      <c r="H10" s="15">
+      <c r="H10" s="6">
         <v>0.48672374094551829</v>
       </c>
-      <c r="I10" s="15">
+      <c r="I10" s="6">
         <v>0.40024992192379</v>
       </c>
-      <c r="J10" s="15">
+      <c r="J10" s="6">
         <v>9.1651513899116799E-2</v>
       </c>
-      <c r="K10" s="15">
+      <c r="K10" s="6">
         <v>2.2360679774997901E-2</v>
       </c>
     </row>
-    <row r="11" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="1">
         <v>7</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="6">
         <v>0.38483762809787708</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="6">
         <v>4.5825756949558413E-2</v>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="6">
         <v>0.1048808848170152</v>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="6">
         <v>0.32078029864690882</v>
       </c>
-      <c r="G11" s="15">
+      <c r="G11" s="6">
         <v>0.10049875621120891</v>
       </c>
-      <c r="H11" s="15">
+      <c r="H11" s="6">
         <v>0.59949979149287447</v>
       </c>
-      <c r="I11" s="15">
+      <c r="I11" s="6">
         <v>0.42953463189829061</v>
       </c>
-      <c r="J11" s="15">
+      <c r="J11" s="6">
         <v>8.306623862918075E-2</v>
       </c>
-      <c r="K11" s="15">
+      <c r="K11" s="6">
         <v>0.02</v>
       </c>
     </row>
-    <row r="12" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="1">
         <v>8</v>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="6">
         <v>2.7133927102430269</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="6">
         <v>2.4821563206212449</v>
       </c>
-      <c r="E12" s="15">
+      <c r="E12" s="6">
         <v>1.2140016474453399</v>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="6">
         <v>4.9240024370424518</v>
       </c>
-      <c r="G12" s="15">
+      <c r="G12" s="6">
         <v>3.040361820573334</v>
       </c>
-      <c r="H12" s="15">
+      <c r="H12" s="6">
         <v>4.3132470367462146</v>
       </c>
-      <c r="I12" s="15">
+      <c r="I12" s="6">
         <v>2.816682445715172</v>
       </c>
-      <c r="J12" s="15">
+      <c r="J12" s="6">
         <v>0.89560035730229592</v>
       </c>
-      <c r="K12" s="15">
+      <c r="K12" s="6">
         <v>2.4326323191144201</v>
+      </c>
+    </row>
+    <row r="14" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="M14" t="s">
+        <v>1</v>
+      </c>
+      <c r="N14" t="s">
+        <v>2</v>
+      </c>
+      <c r="O14" t="s">
+        <v>3</v>
+      </c>
+      <c r="P14" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>5</v>
+      </c>
+      <c r="R14" t="s">
+        <v>6</v>
+      </c>
+      <c r="S14" t="s">
+        <v>7</v>
+      </c>
+      <c r="T14" t="s">
+        <v>8</v>
+      </c>
+      <c r="U14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C15">
+        <v>0.63316664473106921</v>
+      </c>
+      <c r="D15">
+        <v>0.43139309220245969</v>
+      </c>
+      <c r="E15">
+        <v>0.16583123951777001</v>
+      </c>
+      <c r="F15">
+        <v>0.53944415837044712</v>
+      </c>
+      <c r="G15">
+        <v>0.5652433104425032</v>
+      </c>
+      <c r="H15">
+        <v>0.45376205218153709</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0.54525223520862343</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15" s="17">
+        <f>C15-C5</f>
+        <v>0.50906990827116061</v>
+      </c>
+      <c r="N15" s="17">
+        <f t="shared" ref="N15:U22" si="0">D15-D5</f>
+        <v>0.1001831889688759</v>
+      </c>
+      <c r="O15" s="17">
+        <f t="shared" si="0"/>
+        <v>0.1110589837672534</v>
+      </c>
+      <c r="P15" s="17">
+        <f t="shared" si="0"/>
+        <v>0.33844664594802931</v>
+      </c>
+      <c r="Q15" s="17">
+        <f t="shared" si="0"/>
+        <v>0.22085980328805188</v>
+      </c>
+      <c r="R15" s="17">
+        <f t="shared" si="0"/>
+        <v>0.15011752316775762</v>
+      </c>
+      <c r="S15" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.41892720131306832</v>
+      </c>
+      <c r="T15" s="17">
+        <f t="shared" si="0"/>
+        <v>0.42650881433824422</v>
+      </c>
+      <c r="U15" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.40323690307311899</v>
+      </c>
+    </row>
+    <row r="16" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C16">
+        <v>0.15297058540778349</v>
+      </c>
+      <c r="D16">
+        <v>0.232163735324878</v>
+      </c>
+      <c r="E16">
+        <v>0.22494443758403981</v>
+      </c>
+      <c r="F16">
+        <v>6.1644140029689758E-2</v>
+      </c>
+      <c r="G16">
+        <v>0.1367479433117734</v>
+      </c>
+      <c r="H16">
+        <v>0.12569805089976541</v>
+      </c>
+      <c r="I16">
+        <v>0.01</v>
+      </c>
+      <c r="J16">
+        <v>0.4330127018922193</v>
+      </c>
+      <c r="K16">
+        <v>0.01</v>
+      </c>
+      <c r="L16">
+        <v>2</v>
+      </c>
+      <c r="M16" s="17">
+        <f t="shared" ref="M16:M22" si="1">C16-C6</f>
+        <v>8.2259907289128728E-2</v>
+      </c>
+      <c r="N16" s="17">
+        <f t="shared" si="0"/>
+        <v>0.16735632834079939</v>
+      </c>
+      <c r="O16" s="17">
+        <f t="shared" si="0"/>
+        <v>2.5946950162715809E-2</v>
+      </c>
+      <c r="P16" s="17">
+        <f t="shared" si="0"/>
+        <v>-4.3236744787325442E-2</v>
+      </c>
+      <c r="Q16" s="17">
+        <f t="shared" si="0"/>
+        <v>8.5757748175845555E-2</v>
+      </c>
+      <c r="R16" s="17">
+        <f t="shared" si="0"/>
+        <v>-5.4856649952912506E-2</v>
+      </c>
+      <c r="S16" s="17">
+        <f t="shared" si="0"/>
+        <v>-7.5440037453175318E-2</v>
+      </c>
+      <c r="T16" s="17">
+        <f t="shared" si="0"/>
+        <v>0.39178164563604267</v>
+      </c>
+      <c r="U16" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.61233431530006444</v>
+      </c>
+    </row>
+    <row r="17" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C17">
+        <v>0.53347914673396557</v>
+      </c>
+      <c r="D17">
+        <v>0.54744862772683978</v>
+      </c>
+      <c r="E17">
+        <v>0.28583211855912899</v>
+      </c>
+      <c r="F17">
+        <v>0.35594943461115369</v>
+      </c>
+      <c r="G17">
+        <v>0.7058328414008519</v>
+      </c>
+      <c r="H17">
+        <v>0.45398237851264672</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>0.66558245169174945</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>3</v>
+      </c>
+      <c r="M17" s="17">
+        <f t="shared" si="1"/>
+        <v>0.37038408243096466</v>
+      </c>
+      <c r="N17" s="17">
+        <f t="shared" si="0"/>
+        <v>0.11721613244086065</v>
+      </c>
+      <c r="O17" s="17">
+        <f t="shared" si="0"/>
+        <v>0.18734354054116795</v>
+      </c>
+      <c r="P17" s="17">
+        <f t="shared" si="0"/>
+        <v>0.14031084808267538</v>
+      </c>
+      <c r="Q17" s="17">
+        <f t="shared" si="0"/>
+        <v>0.28464404762779821</v>
+      </c>
+      <c r="R17" s="17">
+        <f t="shared" si="0"/>
+        <v>0.31723443520087335</v>
+      </c>
+      <c r="S17" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.35693136595149488</v>
+      </c>
+      <c r="T17" s="17">
+        <f t="shared" si="0"/>
+        <v>0.56608370798108743</v>
+      </c>
+      <c r="U17" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.39522145690739008</v>
+      </c>
+    </row>
+    <row r="18" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C18">
+        <v>0.67230945255886454</v>
+      </c>
+      <c r="D18">
+        <v>0.5487257967327579</v>
+      </c>
+      <c r="E18">
+        <v>0.2215851980616034</v>
+      </c>
+      <c r="F18">
+        <v>0.59110066824526597</v>
+      </c>
+      <c r="G18">
+        <v>0.744983221287567</v>
+      </c>
+      <c r="H18">
+        <v>0.68454364360499331</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0.63079315151640636</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>4</v>
+      </c>
+      <c r="M18" s="17">
+        <f t="shared" si="1"/>
+        <v>0.48336501628195261</v>
+      </c>
+      <c r="N18" s="17">
+        <f t="shared" si="0"/>
+        <v>0.33401669119691901</v>
+      </c>
+      <c r="O18" s="17">
+        <f t="shared" si="0"/>
+        <v>8.4107927212928202E-2</v>
+      </c>
+      <c r="P18" s="17">
+        <f t="shared" si="0"/>
+        <v>0.43878520612798777</v>
+      </c>
+      <c r="Q18" s="17">
+        <f t="shared" si="0"/>
+        <v>0.5677827698208735</v>
+      </c>
+      <c r="R18" s="17">
+        <f t="shared" si="0"/>
+        <v>0.33914532282158244</v>
+      </c>
+      <c r="S18" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.28390139133156778</v>
+      </c>
+      <c r="T18" s="17">
+        <f t="shared" si="0"/>
+        <v>0.54476989884598015</v>
+      </c>
+      <c r="U18" s="17">
+        <f t="shared" si="0"/>
+        <v>-1.094714574672321</v>
+      </c>
+    </row>
+    <row r="19" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <v>0.1606237840420901</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0.13964240043768941</v>
+      </c>
+      <c r="G19">
+        <v>0.21610182784974311</v>
+      </c>
+      <c r="H19">
+        <v>0.26419689627245813</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>0.01</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>5</v>
+      </c>
+      <c r="M19" s="17">
+        <f t="shared" si="1"/>
+        <v>-0.1212435565298214</v>
+      </c>
+      <c r="N19" s="17">
+        <f t="shared" si="0"/>
+        <v>-8.8574931845452093E-2</v>
+      </c>
+      <c r="O19" s="17">
+        <f t="shared" si="0"/>
+        <v>-9.6436507609929556E-2</v>
+      </c>
+      <c r="P19" s="17">
+        <f t="shared" si="0"/>
+        <v>-4.1741171034481078E-2</v>
+      </c>
+      <c r="Q19" s="17">
+        <f t="shared" si="0"/>
+        <v>-7.0079932575340592E-2</v>
+      </c>
+      <c r="R19" s="17">
+        <f t="shared" si="0"/>
+        <v>8.2537875026608615E-2</v>
+      </c>
+      <c r="S19" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.48249352327259282</v>
+      </c>
+      <c r="T19" s="17">
+        <f t="shared" si="0"/>
+        <v>-7.3066238629180755E-2</v>
+      </c>
+      <c r="U19" s="17">
+        <f t="shared" si="0"/>
+        <v>-2.178577517555893</v>
+      </c>
+    </row>
+    <row r="20" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>0.01</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>6</v>
+      </c>
+      <c r="M20" s="17">
+        <f t="shared" si="1"/>
+        <v>-0.41448763552125412</v>
+      </c>
+      <c r="N20" s="17">
+        <f t="shared" si="0"/>
+        <v>-8.0553851381374164E-2</v>
+      </c>
+      <c r="O20" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.10049875621120891</v>
+      </c>
+      <c r="P20" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.2929163703175362</v>
+      </c>
+      <c r="Q20" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.1118033988749895</v>
+      </c>
+      <c r="R20" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.48672374094551829</v>
+      </c>
+      <c r="S20" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.40024992192379</v>
+      </c>
+      <c r="T20" s="17">
+        <f t="shared" si="0"/>
+        <v>-9.1651513899116799E-2</v>
+      </c>
+      <c r="U20" s="17">
+        <f t="shared" si="0"/>
+        <v>-2.2360679774997901E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <v>7</v>
+      </c>
+      <c r="M21" s="17">
+        <f t="shared" si="1"/>
+        <v>-0.38483762809787708</v>
+      </c>
+      <c r="N21" s="17">
+        <f t="shared" si="0"/>
+        <v>-4.5825756949558413E-2</v>
+      </c>
+      <c r="O21" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.1048808848170152</v>
+      </c>
+      <c r="P21" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.32078029864690882</v>
+      </c>
+      <c r="Q21" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.10049875621120891</v>
+      </c>
+      <c r="R21" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.59949979149287447</v>
+      </c>
+      <c r="S21" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.42953463189829061</v>
+      </c>
+      <c r="T21" s="17">
+        <f t="shared" si="0"/>
+        <v>-8.306623862918075E-2</v>
+      </c>
+      <c r="U21" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="22" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C22">
+        <v>1.1156164215356461</v>
+      </c>
+      <c r="D22">
+        <v>0.92493242996448133</v>
+      </c>
+      <c r="E22">
+        <v>0.1667333200053307</v>
+      </c>
+      <c r="F22">
+        <v>2.0715453169071631</v>
+      </c>
+      <c r="G22">
+        <v>1.259880946756478</v>
+      </c>
+      <c r="H22">
+        <v>2.3482333785209679</v>
+      </c>
+      <c r="I22">
+        <v>1.4142135623730951E-2</v>
+      </c>
+      <c r="J22">
+        <v>0.93514704726048303</v>
+      </c>
+      <c r="K22">
+        <v>0.8686195945291586</v>
+      </c>
+      <c r="L22">
+        <v>8</v>
+      </c>
+      <c r="M22" s="17">
+        <f t="shared" si="1"/>
+        <v>-1.5977762887073808</v>
+      </c>
+      <c r="N22" s="17">
+        <f t="shared" si="0"/>
+        <v>-1.5572238906567635</v>
+      </c>
+      <c r="O22" s="17">
+        <f t="shared" si="0"/>
+        <v>-1.0472683274400092</v>
+      </c>
+      <c r="P22" s="17">
+        <f t="shared" si="0"/>
+        <v>-2.8524571201352886</v>
+      </c>
+      <c r="Q22" s="17">
+        <f t="shared" si="0"/>
+        <v>-1.780480873816856</v>
+      </c>
+      <c r="R22" s="17">
+        <f t="shared" si="0"/>
+        <v>-1.9650136582252467</v>
+      </c>
+      <c r="S22" s="17">
+        <f t="shared" si="0"/>
+        <v>-2.802540310091441</v>
+      </c>
+      <c r="T22" s="17">
+        <f t="shared" si="0"/>
+        <v>3.9546689958187109E-2</v>
+      </c>
+      <c r="U22" s="17">
+        <f t="shared" si="0"/>
+        <v>-1.5640127245852615</v>
       </c>
     </row>
   </sheetData>
@@ -1108,10 +1682,22 @@
     <mergeCell ref="B2:K2"/>
   </mergeCells>
   <conditionalFormatting sqref="C5:K12">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M15:U22">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FFF8696B"/>
       </colorScale>
@@ -1131,18 +1717,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="10"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -1460,18 +2046,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="10"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -1789,18 +2375,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="10"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -2128,18 +2714,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="10"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -2467,18 +3053,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="10"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -2796,18 +3382,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="10"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -3125,18 +3711,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:22" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="10"/>
     </row>
     <row r="3" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -3984,18 +4570,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="10"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -4313,18 +4899,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="10"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -4642,18 +5228,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:25" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="10"/>
     </row>
     <row r="3" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
@@ -4953,6 +5539,35 @@
         <v>0.61712734060000018</v>
       </c>
     </row>
+    <row r="14" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="M14" t="s">
+        <v>1</v>
+      </c>
+      <c r="N14" t="s">
+        <v>2</v>
+      </c>
+      <c r="O14" t="s">
+        <v>3</v>
+      </c>
+      <c r="P14" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>5</v>
+      </c>
+      <c r="R14" t="s">
+        <v>6</v>
+      </c>
+      <c r="S14" t="s">
+        <v>7</v>
+      </c>
+      <c r="T14" t="s">
+        <v>8</v>
+      </c>
+      <c r="U14" t="s">
+        <v>9</v>
+      </c>
+    </row>
     <row r="15" spans="2:25" x14ac:dyDescent="0.25">
       <c r="C15">
         <v>0.39257886780000018</v>
@@ -4981,46 +5596,49 @@
       <c r="K15">
         <v>0.31801963179999992</v>
       </c>
-      <c r="M15" s="16">
-        <f>C5-C15</f>
-        <v>4.4517850399999614E-2</v>
-      </c>
-      <c r="N15" s="16">
-        <f t="shared" ref="N15:Y22" si="0">D5-D15</f>
-        <v>3.2599257200000176E-2</v>
-      </c>
-      <c r="O15" s="16">
-        <f t="shared" si="0"/>
-        <v>-8.2913135800000204E-2</v>
-      </c>
-      <c r="P15" s="16">
-        <f t="shared" si="0"/>
-        <v>2.6177366799999824E-2</v>
-      </c>
-      <c r="Q15" s="16">
-        <f t="shared" si="0"/>
-        <v>5.3742515000000157E-2</v>
-      </c>
-      <c r="R15" s="16">
-        <f t="shared" si="0"/>
-        <v>2.1986811199999678E-2</v>
-      </c>
-      <c r="S15" s="16">
-        <f t="shared" si="0"/>
-        <v>-1.1537633600000151E-2</v>
-      </c>
-      <c r="T15" s="16">
-        <f t="shared" si="0"/>
-        <v>8.4355340000022427E-4</v>
-      </c>
-      <c r="U15" s="16">
-        <f t="shared" si="0"/>
-        <v>1.9755476400000249E-2</v>
-      </c>
-      <c r="V15" s="16"/>
-      <c r="W15" s="16"/>
-      <c r="X15" s="16"/>
-      <c r="Y15" s="16"/>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15" s="7">
+        <f>C15-C5</f>
+        <v>-4.4517850399999614E-2</v>
+      </c>
+      <c r="N15" s="7">
+        <f t="shared" ref="N15:U15" si="0">D15-D5</f>
+        <v>-3.2599257200000176E-2</v>
+      </c>
+      <c r="O15" s="7">
+        <f t="shared" si="0"/>
+        <v>8.2913135800000204E-2</v>
+      </c>
+      <c r="P15" s="7">
+        <f t="shared" si="0"/>
+        <v>-2.6177366799999824E-2</v>
+      </c>
+      <c r="Q15" s="7">
+        <f t="shared" si="0"/>
+        <v>-5.3742515000000157E-2</v>
+      </c>
+      <c r="R15" s="7">
+        <f t="shared" si="0"/>
+        <v>-2.1986811199999678E-2</v>
+      </c>
+      <c r="S15" s="7">
+        <f t="shared" si="0"/>
+        <v>1.1537633600000151E-2</v>
+      </c>
+      <c r="T15" s="7">
+        <f t="shared" si="0"/>
+        <v>-8.4355340000022427E-4</v>
+      </c>
+      <c r="U15" s="7">
+        <f t="shared" si="0"/>
+        <v>-1.9755476400000249E-2</v>
+      </c>
+      <c r="V15" s="7"/>
+      <c r="W15" s="7"/>
+      <c r="X15" s="7"/>
+      <c r="Y15" s="7"/>
     </row>
     <row r="16" spans="2:25" x14ac:dyDescent="0.25">
       <c r="C16">
@@ -5050,46 +5668,49 @@
       <c r="K16">
         <v>0.16653376799999989</v>
       </c>
-      <c r="M16" s="16">
-        <f t="shared" ref="M16:M22" si="1">C6-C16</f>
-        <v>7.1810884599999181E-2</v>
-      </c>
-      <c r="N16" s="16">
-        <f t="shared" si="0"/>
-        <v>0.15442469500000033</v>
-      </c>
-      <c r="O16" s="16">
-        <f t="shared" si="0"/>
-        <v>7.1974153000000152E-2</v>
-      </c>
-      <c r="P16" s="16">
-        <f t="shared" si="0"/>
-        <v>9.2137800399999747E-2</v>
-      </c>
-      <c r="Q16" s="16">
-        <f t="shared" si="0"/>
-        <v>0.16386705080000041</v>
-      </c>
-      <c r="R16" s="16">
-        <f t="shared" si="0"/>
-        <v>0.11194769959999995</v>
-      </c>
-      <c r="S16" s="16">
-        <f t="shared" si="0"/>
-        <v>6.1933146399999917E-2</v>
-      </c>
-      <c r="T16" s="16">
-        <f t="shared" si="0"/>
-        <v>0.13812506640000016</v>
-      </c>
-      <c r="U16" s="16">
-        <f t="shared" si="0"/>
-        <v>0.14522724180000021</v>
-      </c>
-      <c r="V16" s="16"/>
-      <c r="W16" s="16"/>
-      <c r="X16" s="16"/>
-      <c r="Y16" s="16"/>
+      <c r="L16">
+        <v>2</v>
+      </c>
+      <c r="M16" s="7">
+        <f t="shared" ref="M16:M22" si="1">C16-C6</f>
+        <v>-7.1810884599999181E-2</v>
+      </c>
+      <c r="N16" s="7">
+        <f t="shared" ref="N16:N22" si="2">D16-D6</f>
+        <v>-0.15442469500000033</v>
+      </c>
+      <c r="O16" s="7">
+        <f t="shared" ref="O16:O22" si="3">E16-E6</f>
+        <v>-7.1974153000000152E-2</v>
+      </c>
+      <c r="P16" s="7">
+        <f t="shared" ref="P16:P22" si="4">F16-F6</f>
+        <v>-9.2137800399999747E-2</v>
+      </c>
+      <c r="Q16" s="7">
+        <f t="shared" ref="Q16:Q22" si="5">G16-G6</f>
+        <v>-0.16386705080000041</v>
+      </c>
+      <c r="R16" s="7">
+        <f t="shared" ref="R16:R22" si="6">H16-H6</f>
+        <v>-0.11194769959999995</v>
+      </c>
+      <c r="S16" s="7">
+        <f t="shared" ref="S16:S22" si="7">I16-I6</f>
+        <v>-6.1933146399999917E-2</v>
+      </c>
+      <c r="T16" s="7">
+        <f t="shared" ref="T16:T22" si="8">J16-J6</f>
+        <v>-0.13812506640000016</v>
+      </c>
+      <c r="U16" s="7">
+        <f t="shared" ref="U16:U22" si="9">K16-K6</f>
+        <v>-0.14522724180000021</v>
+      </c>
+      <c r="V16" s="7"/>
+      <c r="W16" s="7"/>
+      <c r="X16" s="7"/>
+      <c r="Y16" s="7"/>
     </row>
     <row r="17" spans="3:25" x14ac:dyDescent="0.25">
       <c r="C17">
@@ -5119,46 +5740,49 @@
       <c r="K17">
         <v>7.0749640000000724E-4</v>
       </c>
-      <c r="M17" s="16">
+      <c r="L17">
+        <v>3</v>
+      </c>
+      <c r="M17" s="7">
         <f t="shared" si="1"/>
-        <v>4.0327294799999469E-2</v>
-      </c>
-      <c r="N17" s="16">
-        <f t="shared" si="0"/>
-        <v>3.3742135999998979E-3</v>
-      </c>
-      <c r="O17" s="16">
-        <f t="shared" si="0"/>
-        <v>-4.1660653400000136E-2</v>
-      </c>
-      <c r="P17" s="16">
-        <f t="shared" si="0"/>
-        <v>7.3470779999990077E-4</v>
-      </c>
-      <c r="Q17" s="16">
-        <f t="shared" si="0"/>
-        <v>3.57285681999997E-2</v>
-      </c>
-      <c r="R17" s="16">
-        <f t="shared" si="0"/>
-        <v>-1.9483362400000426E-2</v>
-      </c>
-      <c r="S17" s="16">
-        <f t="shared" si="0"/>
-        <v>-3.6191161999994392E-3</v>
-      </c>
-      <c r="T17" s="16">
-        <f t="shared" si="0"/>
-        <v>-2.5633138799999955E-2</v>
-      </c>
-      <c r="U17" s="16">
-        <f t="shared" si="0"/>
-        <v>4.0817100000012374E-4</v>
-      </c>
-      <c r="V17" s="16"/>
-      <c r="W17" s="16"/>
-      <c r="X17" s="16"/>
-      <c r="Y17" s="16"/>
+        <v>-4.0327294799999469E-2</v>
+      </c>
+      <c r="N17" s="7">
+        <f t="shared" si="2"/>
+        <v>-3.3742135999998979E-3</v>
+      </c>
+      <c r="O17" s="7">
+        <f t="shared" si="3"/>
+        <v>4.1660653400000136E-2</v>
+      </c>
+      <c r="P17" s="7">
+        <f t="shared" si="4"/>
+        <v>-7.3470779999990077E-4</v>
+      </c>
+      <c r="Q17" s="7">
+        <f t="shared" si="5"/>
+        <v>-3.57285681999997E-2</v>
+      </c>
+      <c r="R17" s="7">
+        <f t="shared" si="6"/>
+        <v>1.9483362400000426E-2</v>
+      </c>
+      <c r="S17" s="7">
+        <f t="shared" si="7"/>
+        <v>3.6191161999994392E-3</v>
+      </c>
+      <c r="T17" s="7">
+        <f t="shared" si="8"/>
+        <v>2.5633138799999955E-2</v>
+      </c>
+      <c r="U17" s="7">
+        <f t="shared" si="9"/>
+        <v>-4.0817100000012374E-4</v>
+      </c>
+      <c r="V17" s="7"/>
+      <c r="W17" s="7"/>
+      <c r="X17" s="7"/>
+      <c r="Y17" s="7"/>
     </row>
     <row r="18" spans="3:25" x14ac:dyDescent="0.25">
       <c r="C18">
@@ -5188,46 +5812,49 @@
       <c r="K18">
         <v>1.496626999999862E-3</v>
       </c>
-      <c r="M18" s="16">
+      <c r="L18">
+        <v>4</v>
+      </c>
+      <c r="M18" s="7">
         <f t="shared" si="1"/>
-        <v>0.19004441759999985</v>
-      </c>
-      <c r="N18" s="16">
-        <f t="shared" si="0"/>
-        <v>6.6586295799999584E-2</v>
-      </c>
-      <c r="O18" s="16">
-        <f t="shared" si="0"/>
-        <v>-3.0367922399999525E-2</v>
-      </c>
-      <c r="P18" s="16">
-        <f t="shared" si="0"/>
-        <v>0.11083203219999976</v>
-      </c>
-      <c r="Q18" s="16">
-        <f t="shared" si="0"/>
-        <v>8.8926855200000543E-2</v>
-      </c>
-      <c r="R18" s="16">
-        <f t="shared" si="0"/>
-        <v>0.13529508080000019</v>
-      </c>
-      <c r="S18" s="16">
-        <f t="shared" si="0"/>
-        <v>-6.5851588000001016E-3</v>
-      </c>
-      <c r="T18" s="16">
-        <f t="shared" si="0"/>
-        <v>-2.7755627999997146E-3</v>
-      </c>
-      <c r="U18" s="16">
-        <f t="shared" si="0"/>
-        <v>7.8913059999998758E-3</v>
-      </c>
-      <c r="V18" s="16"/>
-      <c r="W18" s="16"/>
-      <c r="X18" s="16"/>
-      <c r="Y18" s="16"/>
+        <v>-0.19004441759999985</v>
+      </c>
+      <c r="N18" s="7">
+        <f t="shared" si="2"/>
+        <v>-6.6586295799999584E-2</v>
+      </c>
+      <c r="O18" s="7">
+        <f t="shared" si="3"/>
+        <v>3.0367922399999525E-2</v>
+      </c>
+      <c r="P18" s="7">
+        <f t="shared" si="4"/>
+        <v>-0.11083203219999976</v>
+      </c>
+      <c r="Q18" s="7">
+        <f t="shared" si="5"/>
+        <v>-8.8926855200000543E-2</v>
+      </c>
+      <c r="R18" s="7">
+        <f t="shared" si="6"/>
+        <v>-0.13529508080000019</v>
+      </c>
+      <c r="S18" s="7">
+        <f t="shared" si="7"/>
+        <v>6.5851588000001016E-3</v>
+      </c>
+      <c r="T18" s="7">
+        <f t="shared" si="8"/>
+        <v>2.7755627999997146E-3</v>
+      </c>
+      <c r="U18" s="7">
+        <f t="shared" si="9"/>
+        <v>-7.8913059999998758E-3</v>
+      </c>
+      <c r="V18" s="7"/>
+      <c r="W18" s="7"/>
+      <c r="X18" s="7"/>
+      <c r="Y18" s="7"/>
     </row>
     <row r="19" spans="3:25" x14ac:dyDescent="0.25">
       <c r="C19">
@@ -5257,46 +5884,49 @@
       <c r="K19">
         <v>4.2939589200000412E-2</v>
       </c>
-      <c r="M19" s="16">
+      <c r="L19">
+        <v>5</v>
+      </c>
+      <c r="M19" s="7">
         <f t="shared" si="1"/>
-        <v>1.3714545600000072E-2</v>
-      </c>
-      <c r="N19" s="16">
-        <f t="shared" si="0"/>
-        <v>1.2245130000000215E-2</v>
-      </c>
-      <c r="O19" s="16">
-        <f t="shared" si="0"/>
-        <v>-3.2653679999983254E-4</v>
-      </c>
-      <c r="P19" s="16">
-        <f t="shared" si="0"/>
-        <v>4.4055256599999981E-2</v>
-      </c>
-      <c r="Q19" s="16">
-        <f t="shared" si="0"/>
-        <v>2.4680739800000406E-2</v>
-      </c>
-      <c r="R19" s="16">
-        <f t="shared" si="0"/>
-        <v>1.9456150999999644E-2</v>
-      </c>
-      <c r="S19" s="16">
-        <f t="shared" si="0"/>
-        <v>-2.7211399999504938E-5</v>
-      </c>
-      <c r="T19" s="16">
-        <f t="shared" si="0"/>
-        <v>1.3605700000018928E-4</v>
-      </c>
-      <c r="U19" s="16">
-        <f>K9-K19</f>
-        <v>-4.3266126000003416E-3</v>
-      </c>
-      <c r="V19" s="16"/>
-      <c r="W19" s="16"/>
-      <c r="X19" s="16"/>
-      <c r="Y19" s="16"/>
+        <v>-1.3714545600000072E-2</v>
+      </c>
+      <c r="N19" s="7">
+        <f t="shared" si="2"/>
+        <v>-1.2245130000000215E-2</v>
+      </c>
+      <c r="O19" s="7">
+        <f t="shared" si="3"/>
+        <v>3.2653679999983254E-4</v>
+      </c>
+      <c r="P19" s="7">
+        <f t="shared" si="4"/>
+        <v>-4.4055256599999981E-2</v>
+      </c>
+      <c r="Q19" s="7">
+        <f t="shared" si="5"/>
+        <v>-2.4680739800000406E-2</v>
+      </c>
+      <c r="R19" s="7">
+        <f t="shared" si="6"/>
+        <v>-1.9456150999999644E-2</v>
+      </c>
+      <c r="S19" s="7">
+        <f t="shared" si="7"/>
+        <v>2.7211399999504938E-5</v>
+      </c>
+      <c r="T19" s="7">
+        <f t="shared" si="8"/>
+        <v>-1.3605700000018928E-4</v>
+      </c>
+      <c r="U19" s="7">
+        <f t="shared" si="9"/>
+        <v>4.3266126000003416E-3</v>
+      </c>
+      <c r="V19" s="7"/>
+      <c r="W19" s="7"/>
+      <c r="X19" s="7"/>
+      <c r="Y19" s="7"/>
     </row>
     <row r="20" spans="3:25" x14ac:dyDescent="0.25">
       <c r="C20">
@@ -5326,46 +5956,49 @@
       <c r="K20">
         <v>2.7211399999949041E-5</v>
       </c>
-      <c r="M20" s="16">
+      <c r="L20">
+        <v>6</v>
+      </c>
+      <c r="M20" s="7">
         <f t="shared" si="1"/>
-        <v>9.9131130199999945E-2</v>
-      </c>
-      <c r="N20" s="16">
-        <f t="shared" si="0"/>
-        <v>6.6014856399999794E-2</v>
-      </c>
-      <c r="O20" s="16">
-        <f t="shared" si="0"/>
-        <v>-1.25172440000032E-3</v>
-      </c>
-      <c r="P20" s="16">
-        <f t="shared" si="0"/>
-        <v>9.3035776599999898E-2</v>
-      </c>
-      <c r="Q20" s="16">
-        <f t="shared" si="0"/>
-        <v>0.10974357619999919</v>
-      </c>
-      <c r="R20" s="16">
-        <f t="shared" si="0"/>
-        <v>7.3960585199999651E-2</v>
-      </c>
-      <c r="S20" s="16">
-        <f t="shared" si="0"/>
+        <v>-9.9131130199999945E-2</v>
+      </c>
+      <c r="N20" s="7">
+        <f t="shared" si="2"/>
+        <v>-6.6014856399999794E-2</v>
+      </c>
+      <c r="O20" s="7">
+        <f t="shared" si="3"/>
+        <v>1.25172440000032E-3</v>
+      </c>
+      <c r="P20" s="7">
+        <f t="shared" si="4"/>
+        <v>-9.3035776599999898E-2</v>
+      </c>
+      <c r="Q20" s="7">
+        <f t="shared" si="5"/>
+        <v>-0.10974357619999919</v>
+      </c>
+      <c r="R20" s="7">
+        <f t="shared" si="6"/>
+        <v>-7.3960585199999651E-2</v>
+      </c>
+      <c r="S20" s="7">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="T20" s="16">
-        <f t="shared" si="0"/>
-        <v>2.8299855999995849E-3</v>
-      </c>
-      <c r="U20" s="16">
-        <f t="shared" si="0"/>
-        <v>-2.7211399999949041E-5</v>
-      </c>
-      <c r="V20" s="16"/>
-      <c r="W20" s="16"/>
-      <c r="X20" s="16"/>
-      <c r="Y20" s="16"/>
+      <c r="T20" s="7">
+        <f t="shared" si="8"/>
+        <v>-2.8299855999995849E-3</v>
+      </c>
+      <c r="U20" s="7">
+        <f t="shared" si="9"/>
+        <v>2.7211399999949041E-5</v>
+      </c>
+      <c r="V20" s="7"/>
+      <c r="W20" s="7"/>
+      <c r="X20" s="7"/>
+      <c r="Y20" s="7"/>
     </row>
     <row r="21" spans="3:25" x14ac:dyDescent="0.25">
       <c r="C21">
@@ -5395,46 +6028,49 @@
       <c r="K21">
         <v>2.721140000039313E-5</v>
       </c>
-      <c r="M21" s="16">
+      <c r="L21">
+        <v>7</v>
+      </c>
+      <c r="M21" s="7">
         <f t="shared" si="1"/>
-        <v>4.9660805000000224E-2</v>
-      </c>
-      <c r="N21" s="16">
-        <f t="shared" si="0"/>
-        <v>2.829985600000029E-2</v>
-      </c>
-      <c r="O21" s="16">
-        <f t="shared" si="0"/>
-        <v>-7.3470779999995628E-4</v>
-      </c>
-      <c r="P21" s="16">
-        <f t="shared" si="0"/>
-        <v>6.2885545399999507E-2</v>
-      </c>
-      <c r="Q21" s="16">
-        <f t="shared" si="0"/>
-        <v>8.6967634399999633E-2</v>
-      </c>
-      <c r="R21" s="16">
-        <f t="shared" si="0"/>
-        <v>6.8545516600000383E-2</v>
-      </c>
-      <c r="S21" s="16">
-        <f t="shared" si="0"/>
-        <v>-2.7211400000393117E-5</v>
-      </c>
-      <c r="T21" s="16">
-        <f t="shared" si="0"/>
-        <v>3.8095959999973061E-4</v>
-      </c>
-      <c r="U21" s="16">
-        <f t="shared" si="0"/>
-        <v>-2.721140000039313E-5</v>
-      </c>
-      <c r="V21" s="16"/>
-      <c r="W21" s="16"/>
-      <c r="X21" s="16"/>
-      <c r="Y21" s="16"/>
+        <v>-4.9660805000000224E-2</v>
+      </c>
+      <c r="N21" s="7">
+        <f t="shared" si="2"/>
+        <v>-2.829985600000029E-2</v>
+      </c>
+      <c r="O21" s="7">
+        <f t="shared" si="3"/>
+        <v>7.3470779999995628E-4</v>
+      </c>
+      <c r="P21" s="7">
+        <f t="shared" si="4"/>
+        <v>-6.2885545399999507E-2</v>
+      </c>
+      <c r="Q21" s="7">
+        <f t="shared" si="5"/>
+        <v>-8.6967634399999633E-2</v>
+      </c>
+      <c r="R21" s="7">
+        <f t="shared" si="6"/>
+        <v>-6.8545516600000383E-2</v>
+      </c>
+      <c r="S21" s="7">
+        <f t="shared" si="7"/>
+        <v>2.7211400000393117E-5</v>
+      </c>
+      <c r="T21" s="7">
+        <f t="shared" si="8"/>
+        <v>-3.8095959999973061E-4</v>
+      </c>
+      <c r="U21" s="7">
+        <f t="shared" si="9"/>
+        <v>2.721140000039313E-5</v>
+      </c>
+      <c r="V21" s="7"/>
+      <c r="W21" s="7"/>
+      <c r="X21" s="7"/>
+      <c r="Y21" s="7"/>
     </row>
     <row r="22" spans="3:25" x14ac:dyDescent="0.25">
       <c r="C22">
@@ -5464,46 +6100,49 @@
       <c r="K22">
         <v>0.46240332020000002</v>
       </c>
-      <c r="M22" s="16">
+      <c r="L22">
+        <v>8</v>
+      </c>
+      <c r="M22" s="7">
         <f t="shared" si="1"/>
-        <v>6.7593117599999974E-2</v>
-      </c>
-      <c r="N22" s="16">
-        <f t="shared" si="0"/>
-        <v>7.5484423600000294E-2</v>
-      </c>
-      <c r="O22" s="16">
-        <f t="shared" si="0"/>
-        <v>2.8952929599999622E-2</v>
-      </c>
-      <c r="P22" s="16">
-        <f t="shared" si="0"/>
-        <v>3.7225195200000005E-2</v>
-      </c>
-      <c r="Q22" s="16">
-        <f t="shared" si="0"/>
-        <v>0.12702281519999969</v>
-      </c>
-      <c r="R22" s="16">
-        <f t="shared" si="0"/>
-        <v>7.1048965399999719E-2</v>
-      </c>
-      <c r="S22" s="16">
-        <f t="shared" si="0"/>
-        <v>8.9797620000010153E-4</v>
-      </c>
-      <c r="T22" s="16">
-        <f t="shared" si="0"/>
-        <v>5.9402486199999771E-2</v>
-      </c>
-      <c r="U22" s="16">
-        <f t="shared" si="0"/>
-        <v>0.15472402040000016</v>
-      </c>
-      <c r="V22" s="16"/>
-      <c r="W22" s="16"/>
-      <c r="X22" s="16"/>
-      <c r="Y22" s="16"/>
+        <v>-6.7593117599999974E-2</v>
+      </c>
+      <c r="N22" s="7">
+        <f t="shared" si="2"/>
+        <v>-7.5484423600000294E-2</v>
+      </c>
+      <c r="O22" s="7">
+        <f t="shared" si="3"/>
+        <v>-2.8952929599999622E-2</v>
+      </c>
+      <c r="P22" s="7">
+        <f t="shared" si="4"/>
+        <v>-3.7225195200000005E-2</v>
+      </c>
+      <c r="Q22" s="7">
+        <f t="shared" si="5"/>
+        <v>-0.12702281519999969</v>
+      </c>
+      <c r="R22" s="7">
+        <f t="shared" si="6"/>
+        <v>-7.1048965399999719E-2</v>
+      </c>
+      <c r="S22" s="7">
+        <f t="shared" si="7"/>
+        <v>-8.9797620000010153E-4</v>
+      </c>
+      <c r="T22" s="7">
+        <f t="shared" si="8"/>
+        <v>-5.9402486199999771E-2</v>
+      </c>
+      <c r="U22" s="7">
+        <f t="shared" si="9"/>
+        <v>-0.15472402040000016</v>
+      </c>
+      <c r="V22" s="7"/>
+      <c r="W22" s="7"/>
+      <c r="X22" s="7"/>
+      <c r="Y22" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5538,27 +6177,27 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:K12"/>
+  <dimension ref="B2:U22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="11" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="6" t="s">
+    <row r="2" spans="2:21" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
-    </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="10"/>
+    </row>
+    <row r="3" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -5570,7 +6209,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
     </row>
-    <row r="4" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2"/>
       <c r="C4" s="1" t="s">
         <v>1</v>
@@ -5600,7 +6239,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1">
         <v>1</v>
       </c>
@@ -5632,7 +6271,7 @@
         <v>0.80251860880000025</v>
       </c>
     </row>
-    <row r="6" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <v>2</v>
       </c>
@@ -5664,7 +6303,7 @@
         <v>0.36566679320000001</v>
       </c>
     </row>
-    <row r="7" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="1">
         <v>3</v>
       </c>
@@ -5696,7 +6335,7 @@
         <v>0.86597559360000043</v>
       </c>
     </row>
-    <row r="8" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="1">
         <v>4</v>
       </c>
@@ -5728,7 +6367,7 @@
         <v>0.78978367359999968</v>
       </c>
     </row>
-    <row r="9" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="1">
         <v>5</v>
       </c>
@@ -5760,7 +6399,7 @@
         <v>0.79568854740000017</v>
       </c>
     </row>
-    <row r="10" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1">
         <v>6</v>
       </c>
@@ -5792,7 +6431,7 @@
         <v>0.90646615679999964</v>
       </c>
     </row>
-    <row r="11" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="1">
         <v>7</v>
       </c>
@@ -5824,7 +6463,7 @@
         <v>0.9187929210000001</v>
       </c>
     </row>
-    <row r="12" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="1">
         <v>8</v>
       </c>
@@ -5854,6 +6493,579 @@
       </c>
       <c r="K12" s="5">
         <v>0.86243811160000083</v>
+      </c>
+    </row>
+    <row r="14" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="M14" t="s">
+        <v>1</v>
+      </c>
+      <c r="N14" t="s">
+        <v>2</v>
+      </c>
+      <c r="O14" t="s">
+        <v>3</v>
+      </c>
+      <c r="P14" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>5</v>
+      </c>
+      <c r="R14" t="s">
+        <v>6</v>
+      </c>
+      <c r="S14" t="s">
+        <v>7</v>
+      </c>
+      <c r="T14" t="s">
+        <v>8</v>
+      </c>
+      <c r="U14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C15">
+        <v>0.41437519920000021</v>
+      </c>
+      <c r="D15">
+        <v>0.49619987899999968</v>
+      </c>
+      <c r="E15">
+        <v>0.23037171239999979</v>
+      </c>
+      <c r="F15">
+        <v>0.54371098340000046</v>
+      </c>
+      <c r="G15">
+        <v>0.57595649239999958</v>
+      </c>
+      <c r="H15">
+        <v>0.68439392140000033</v>
+      </c>
+      <c r="I15">
+        <v>1.7524141599999599E-2</v>
+      </c>
+      <c r="J15">
+        <v>0.30865891019999969</v>
+      </c>
+      <c r="K15">
+        <v>0.31845501419999961</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15" s="7">
+        <f>C15-C5</f>
+        <v>-0.1475402107999999</v>
+      </c>
+      <c r="N15" s="7">
+        <f t="shared" ref="N15:U22" si="0">D15-D5</f>
+        <v>-0.16598954000000049</v>
+      </c>
+      <c r="O15" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.10326726300000019</v>
+      </c>
+      <c r="P15" s="7">
+        <f t="shared" si="0"/>
+        <v>-8.0545743999999697E-2</v>
+      </c>
+      <c r="Q15" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.11254635040000061</v>
+      </c>
+      <c r="R15" s="7">
+        <f t="shared" si="0"/>
+        <v>-9.8913438999999492E-2</v>
+      </c>
+      <c r="S15" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.40740908080000038</v>
+      </c>
+      <c r="T15" s="7">
+        <f t="shared" si="0"/>
+        <v>2.092556659999989E-2</v>
+      </c>
+      <c r="U15" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.48406359460000065</v>
+      </c>
+    </row>
+    <row r="16" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C16">
+        <v>0.62485537820000037</v>
+      </c>
+      <c r="D16">
+        <v>0.62880103120000008</v>
+      </c>
+      <c r="E16">
+        <v>0.38368074000000002</v>
+      </c>
+      <c r="F16">
+        <v>0.65269264039999975</v>
+      </c>
+      <c r="G16">
+        <v>0.66945486279999944</v>
+      </c>
+      <c r="H16">
+        <v>0.68692458160000003</v>
+      </c>
+      <c r="I16">
+        <v>3.2789737000000319E-2</v>
+      </c>
+      <c r="J16">
+        <v>0.43018502259999991</v>
+      </c>
+      <c r="K16">
+        <v>0.1670507846000002</v>
+      </c>
+      <c r="L16">
+        <v>2</v>
+      </c>
+      <c r="M16" s="7">
+        <f t="shared" ref="M16:M22" si="1">C16-C6</f>
+        <v>-0.33173417739999911</v>
+      </c>
+      <c r="N16" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.13679170780000005</v>
+      </c>
+      <c r="O16" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.11088645500000011</v>
+      </c>
+      <c r="P16" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.24803191100000044</v>
+      </c>
+      <c r="Q16" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.13344470560000055</v>
+      </c>
+      <c r="R16" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.24103858119999977</v>
+      </c>
+      <c r="S16" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.13309095739999949</v>
+      </c>
+      <c r="T16" s="7">
+        <f t="shared" si="0"/>
+        <v>-7.5157886800000462E-2</v>
+      </c>
+      <c r="U16" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.19861600859999981</v>
+      </c>
+    </row>
+    <row r="17" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C17">
+        <v>0.40378996460000011</v>
+      </c>
+      <c r="D17">
+        <v>0.2777467598000003</v>
+      </c>
+      <c r="E17">
+        <v>5.6953460200000361E-2</v>
+      </c>
+      <c r="F17">
+        <v>0.41793989259999981</v>
+      </c>
+      <c r="G17">
+        <v>0.34340786800000028</v>
+      </c>
+      <c r="H17">
+        <v>0.45872978119999969</v>
+      </c>
+      <c r="I17">
+        <v>6.1225650000000797E-3</v>
+      </c>
+      <c r="J17">
+        <v>0.18155446079999971</v>
+      </c>
+      <c r="K17">
+        <v>9.5239899999999267E-4</v>
+      </c>
+      <c r="L17">
+        <v>3</v>
+      </c>
+      <c r="M17" s="7">
+        <f t="shared" si="1"/>
+        <v>-9.2627605600000107E-2</v>
+      </c>
+      <c r="N17" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.13812506640000022</v>
+      </c>
+      <c r="O17" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.14275100439999955</v>
+      </c>
+      <c r="P17" s="7">
+        <f t="shared" si="0"/>
+        <v>-2.9687637400000799E-2</v>
+      </c>
+      <c r="Q17" s="7">
+        <f t="shared" si="0"/>
+        <v>-6.4899188999999691E-2</v>
+      </c>
+      <c r="R17" s="7">
+        <f t="shared" si="0"/>
+        <v>-8.4382551400000116E-2</v>
+      </c>
+      <c r="S17" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.77261328019999986</v>
+      </c>
+      <c r="T17" s="7">
+        <f t="shared" si="0"/>
+        <v>6.8164556999999806E-2</v>
+      </c>
+      <c r="U17" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.86502319460000043</v>
+      </c>
+    </row>
+    <row r="18" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C18">
+        <v>0.55813302540000009</v>
+      </c>
+      <c r="D18">
+        <v>0.34055067100000042</v>
+      </c>
+      <c r="E18">
+        <v>0.11355317219999959</v>
+      </c>
+      <c r="F18">
+        <v>0.52664943560000044</v>
+      </c>
+      <c r="G18">
+        <v>0.42637542660000038</v>
+      </c>
+      <c r="H18">
+        <v>0.58806556539999955</v>
+      </c>
+      <c r="I18">
+        <v>1.687106799999993E-2</v>
+      </c>
+      <c r="J18">
+        <v>0.25249458060000007</v>
+      </c>
+      <c r="K18">
+        <v>1.2245129999999721E-2</v>
+      </c>
+      <c r="L18">
+        <v>4</v>
+      </c>
+      <c r="M18" s="7">
+        <f t="shared" si="1"/>
+        <v>-8.6804365999999966E-2</v>
+      </c>
+      <c r="N18" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.33004707059999955</v>
+      </c>
+      <c r="O18" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.15445190640000028</v>
+      </c>
+      <c r="P18" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.1179342075999994</v>
+      </c>
+      <c r="Q18" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.20101061180000013</v>
+      </c>
+      <c r="R18" s="7">
+        <f t="shared" si="0"/>
+        <v>-9.9212764400000708E-2</v>
+      </c>
+      <c r="S18" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.68091086220000019</v>
+      </c>
+      <c r="T18" s="7">
+        <f t="shared" si="0"/>
+        <v>5.3660880799999866E-2</v>
+      </c>
+      <c r="U18" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.77753854359999997</v>
+      </c>
+    </row>
+    <row r="19" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C19">
+        <v>5.1320700400000252E-2</v>
+      </c>
+      <c r="D19">
+        <v>0.17486045640000031</v>
+      </c>
+      <c r="E19">
+        <v>4.1905556000001454E-3</v>
+      </c>
+      <c r="F19">
+        <v>0.15238384000000019</v>
+      </c>
+      <c r="G19">
+        <v>0.26800507860000028</v>
+      </c>
+      <c r="H19">
+        <v>0.3292035172000003</v>
+      </c>
+      <c r="I19">
+        <v>1.5510497999997601E-3</v>
+      </c>
+      <c r="J19">
+        <v>5.115743200000189E-3</v>
+      </c>
+      <c r="K19">
+        <v>4.3402182999999983E-2</v>
+      </c>
+      <c r="L19">
+        <v>5</v>
+      </c>
+      <c r="M19" s="7">
+        <f t="shared" si="1"/>
+        <v>-0.18032994779999975</v>
+      </c>
+      <c r="N19" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.13145827339999927</v>
+      </c>
+      <c r="O19" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.19178594720000006</v>
+      </c>
+      <c r="P19" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.16188061860000011</v>
+      </c>
+      <c r="Q19" s="7">
+        <f t="shared" si="0"/>
+        <v>-7.8096717999999898E-2</v>
+      </c>
+      <c r="R19" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.17129576299999982</v>
+      </c>
+      <c r="S19" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.66433911960000058</v>
+      </c>
+      <c r="T19" s="7">
+        <f t="shared" si="0"/>
+        <v>-2.5088910800000089E-2</v>
+      </c>
+      <c r="U19" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.75228636440000018</v>
+      </c>
+    </row>
+    <row r="20" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C20">
+        <v>0.1201383309999997</v>
+      </c>
+      <c r="D20">
+        <v>0.14658781179999991</v>
+      </c>
+      <c r="E20">
+        <v>6.0409307999997894E-3</v>
+      </c>
+      <c r="F20">
+        <v>0.19706495880000041</v>
+      </c>
+      <c r="G20">
+        <v>0.21619457300000011</v>
+      </c>
+      <c r="H20">
+        <v>0.28925718200000011</v>
+      </c>
+      <c r="I20">
+        <v>5.2245888000004292E-3</v>
+      </c>
+      <c r="J20">
+        <v>4.7347836000004584E-3</v>
+      </c>
+      <c r="K20">
+        <v>3.8912301999993741E-3</v>
+      </c>
+      <c r="L20">
+        <v>6</v>
+      </c>
+      <c r="M20" s="7">
+        <f t="shared" si="1"/>
+        <v>-0.27682157220000031</v>
+      </c>
+      <c r="N20" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.1485742439999998</v>
+      </c>
+      <c r="O20" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.1915410445999996</v>
+      </c>
+      <c r="P20" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.23793648159999886</v>
+      </c>
+      <c r="Q20" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.11828795579999957</v>
+      </c>
+      <c r="R20" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.28397817039999967</v>
+      </c>
+      <c r="S20" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.69424444819999964</v>
+      </c>
+      <c r="T20" s="7">
+        <f t="shared" si="0"/>
+        <v>-2.639505799999986E-2</v>
+      </c>
+      <c r="U20" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.90257492660000027</v>
+      </c>
+    </row>
+    <row r="21" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C21">
+        <v>6.7266580799999698E-2</v>
+      </c>
+      <c r="D21">
+        <v>6.3647464600000259E-2</v>
+      </c>
+      <c r="E21">
+        <v>1.697991359999973E-2</v>
+      </c>
+      <c r="F21">
+        <v>0.1146144168000003</v>
+      </c>
+      <c r="G21">
+        <v>9.6382778800000235E-2</v>
+      </c>
+      <c r="H21">
+        <v>0.1853368453999997</v>
+      </c>
+      <c r="I21">
+        <v>2.1333737600000461E-2</v>
+      </c>
+      <c r="J21">
+        <v>1.175532480000019E-2</v>
+      </c>
+      <c r="K21">
+        <v>6.0409308000002326E-3</v>
+      </c>
+      <c r="L21">
+        <v>7</v>
+      </c>
+      <c r="M21" s="7">
+        <f t="shared" si="1"/>
+        <v>-0.23521534160000002</v>
+      </c>
+      <c r="N21" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.11665527179999954</v>
+      </c>
+      <c r="O21" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.17638429480000048</v>
+      </c>
+      <c r="P21" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.20092897759999984</v>
+      </c>
+      <c r="Q21" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.11951246879999958</v>
+      </c>
+      <c r="R21" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.2382902298000005</v>
+      </c>
+      <c r="S21" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.68959129879999947</v>
+      </c>
+      <c r="T21" s="7">
+        <f t="shared" si="0"/>
+        <v>-1.8041158199999963E-2</v>
+      </c>
+      <c r="U21" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.91275199019999986</v>
+      </c>
+    </row>
+    <row r="22" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C22">
+        <v>0.67544137079999977</v>
+      </c>
+      <c r="D22">
+        <v>0.63870598080000018</v>
+      </c>
+      <c r="E22">
+        <v>0.37067369080000029</v>
+      </c>
+      <c r="F22">
+        <v>0.71489790080000049</v>
+      </c>
+      <c r="G22">
+        <v>0.69658462860000059</v>
+      </c>
+      <c r="H22">
+        <v>0.81590661760000005</v>
+      </c>
+      <c r="I22">
+        <v>5.5075873599999881E-2</v>
+      </c>
+      <c r="J22">
+        <v>0.45995429419999972</v>
+      </c>
+      <c r="K22">
+        <v>0.48077101519999982</v>
+      </c>
+      <c r="L22">
+        <v>8</v>
+      </c>
+      <c r="M22" s="7">
+        <f t="shared" si="1"/>
+        <v>-0.10881838860000004</v>
+      </c>
+      <c r="N22" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.19777245519999997</v>
+      </c>
+      <c r="O22" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.18607155319999974</v>
+      </c>
+      <c r="P22" s="7">
+        <f t="shared" si="0"/>
+        <v>-7.0858485599999632E-2</v>
+      </c>
+      <c r="Q22" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.18384021840000031</v>
+      </c>
+      <c r="R22" s="7">
+        <f t="shared" si="0"/>
+        <v>-8.5090047800000068E-2</v>
+      </c>
+      <c r="S22" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.31486310939999962</v>
+      </c>
+      <c r="T22" s="7">
+        <f t="shared" si="0"/>
+        <v>-3.7415675000000093E-2</v>
+      </c>
+      <c r="U22" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.38166709640000102</v>
       </c>
     </row>
   </sheetData>
@@ -5861,12 +7073,24 @@
     <mergeCell ref="B2:K2"/>
   </mergeCells>
   <conditionalFormatting sqref="C5:K12">
-    <cfRule type="colorScale" priority="1">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF63BE7B"/>
         <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M15:U22">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -5877,27 +7101,27 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:K12"/>
+  <dimension ref="B2:U22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="11" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="6" t="s">
+    <row r="2" spans="2:21" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
-    </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="10"/>
+    </row>
+    <row r="3" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -5909,7 +7133,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
     </row>
-    <row r="4" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2"/>
       <c r="C4" s="1" t="s">
         <v>1</v>
@@ -5939,260 +7163,833 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1">
         <v>1</v>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="6">
         <v>0.48703182647543691</v>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="6">
         <v>7.5498344352707511E-2</v>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="6">
         <v>0.15427248620541509</v>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="6">
         <v>0.45738386504117079</v>
       </c>
-      <c r="G5" s="15">
+      <c r="G5" s="6">
         <v>7.2801098892805186E-2</v>
       </c>
-      <c r="H5" s="15">
+      <c r="H5" s="6">
         <v>0.33674916480965472</v>
       </c>
-      <c r="I5" s="15">
+      <c r="I5" s="6">
         <v>4.3588989435406733E-2</v>
       </c>
-      <c r="J5" s="15">
+      <c r="J5" s="6">
         <v>0.16643316977093239</v>
       </c>
-      <c r="K5" s="15">
+      <c r="K5" s="6">
         <v>0.17464249196572981</v>
       </c>
     </row>
-    <row r="6" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <v>2</v>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="6">
         <v>9.4339811320566042E-2</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="6">
         <v>0.1532970971675589</v>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="6">
         <v>0.32588341473600652</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="6">
         <v>7.8740078740118111E-2</v>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="6">
         <v>9.1651513899116813E-2</v>
       </c>
-      <c r="H6" s="15">
+      <c r="H6" s="6">
         <v>0.14177446878757829</v>
       </c>
-      <c r="I6" s="15">
+      <c r="I6" s="6">
         <v>0.37229020937972568</v>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="6">
         <v>2.2360679774997901E-2</v>
       </c>
-      <c r="K6" s="15">
+      <c r="K6" s="6">
         <v>0.75352504935138021</v>
       </c>
     </row>
-    <row r="7" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="1">
         <v>3</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="6">
         <v>0.33674916480965472</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="6">
         <v>0.17291616465790591</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="6">
         <v>0.122065556157337</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="6">
         <v>0.37589892258425012</v>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="6">
         <v>7.211102550927978E-2</v>
       </c>
-      <c r="H7" s="15">
+      <c r="H7" s="6">
         <v>0.42860237983473681</v>
       </c>
-      <c r="I7" s="15">
+      <c r="I7" s="6">
         <v>1.4142135623730951E-2</v>
       </c>
-      <c r="J7" s="15">
+      <c r="J7" s="6">
         <v>5.0990195135927847E-2</v>
       </c>
-      <c r="K7" s="15">
+      <c r="K7" s="6">
         <v>0.01</v>
       </c>
     </row>
-    <row r="8" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="1">
         <v>4</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="6">
         <v>0.122065556157337</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="6">
         <v>0.18110770276274829</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="6">
         <v>0.31208973068654472</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="6">
         <v>0.1824828759089466</v>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="6">
         <v>4.8989794855663557E-2</v>
       </c>
-      <c r="H8" s="15">
+      <c r="H8" s="6">
         <v>0.34727510708370679</v>
       </c>
-      <c r="I8" s="15">
+      <c r="I8" s="6">
         <v>3.605551275463989E-2</v>
       </c>
-      <c r="J8" s="15">
+      <c r="J8" s="6">
         <v>1.732050807568877E-2</v>
       </c>
-      <c r="K8" s="15">
+      <c r="K8" s="6">
         <v>0.11</v>
       </c>
     </row>
-    <row r="9" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="1">
         <v>5</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="6">
         <v>0.14071247279470289</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="6">
         <v>0.1729161646579058</v>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="6">
         <v>0</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="6">
         <v>0.39153543900903792</v>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="6">
         <v>0.17464249196572981</v>
       </c>
-      <c r="H9" s="15">
+      <c r="H9" s="6">
         <v>0.34073450074801642</v>
       </c>
-      <c r="I9" s="15">
+      <c r="I9" s="6">
         <v>0</v>
       </c>
-      <c r="J9" s="15">
+      <c r="J9" s="6">
         <v>0</v>
       </c>
-      <c r="K9" s="15">
+      <c r="K9" s="6">
         <v>2.2360679774997901E-2</v>
       </c>
     </row>
-    <row r="10" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1">
         <v>6</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="6">
         <v>5.0990195135927847E-2</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="6">
         <v>0.16763054614240211</v>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="6">
         <v>1.4142135623730951E-2</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="6">
         <v>0.08</v>
       </c>
-      <c r="G10" s="15">
+      <c r="G10" s="6">
         <v>0.24331050121192879</v>
       </c>
-      <c r="H10" s="15">
+      <c r="H10" s="6">
         <v>0.102469507659596</v>
       </c>
-      <c r="I10" s="15">
+      <c r="I10" s="6">
         <v>0</v>
       </c>
-      <c r="J10" s="15">
+      <c r="J10" s="6">
         <v>3.1622776601683791E-2</v>
       </c>
-      <c r="K10" s="15">
+      <c r="K10" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="1">
         <v>7</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="6">
         <v>0.01</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="6">
         <v>0.19339079605813719</v>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="6">
         <v>0</v>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="6">
         <v>0</v>
       </c>
-      <c r="G11" s="15">
+      <c r="G11" s="6">
         <v>0.27294688127912359</v>
       </c>
-      <c r="H11" s="15">
+      <c r="H11" s="6">
         <v>0.01</v>
       </c>
-      <c r="I11" s="15">
+      <c r="I11" s="6">
         <v>0</v>
       </c>
-      <c r="J11" s="15">
+      <c r="J11" s="6">
         <v>0.01</v>
       </c>
-      <c r="K11" s="15">
+      <c r="K11" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="1">
         <v>8</v>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="6">
         <v>3.819698941016163</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="6">
         <v>0.96067684472979764</v>
       </c>
-      <c r="E12" s="15">
+      <c r="E12" s="6">
         <v>0.43023249528597901</v>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="6">
         <v>1.0811567878897119</v>
       </c>
-      <c r="G12" s="15">
+      <c r="G12" s="6">
         <v>1.689289791598825</v>
       </c>
-      <c r="H12" s="15">
+      <c r="H12" s="6">
         <v>1.51175394823364</v>
       </c>
-      <c r="I12" s="15">
+      <c r="I12" s="6">
         <v>0.23622023622035429</v>
       </c>
-      <c r="J12" s="15">
+      <c r="J12" s="6">
         <v>1.157713263291045</v>
       </c>
-      <c r="K12" s="15">
+      <c r="K12" s="6">
         <v>0.41484937025383078</v>
+      </c>
+    </row>
+    <row r="14" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="M14" t="s">
+        <v>1</v>
+      </c>
+      <c r="N14" t="s">
+        <v>2</v>
+      </c>
+      <c r="O14" t="s">
+        <v>3</v>
+      </c>
+      <c r="P14" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>5</v>
+      </c>
+      <c r="R14" t="s">
+        <v>6</v>
+      </c>
+      <c r="S14" t="s">
+        <v>7</v>
+      </c>
+      <c r="T14" t="s">
+        <v>8</v>
+      </c>
+      <c r="U14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C15">
+        <v>5.7445626465380289E-2</v>
+      </c>
+      <c r="D15">
+        <v>7.3484692283495343E-2</v>
+      </c>
+      <c r="E15">
+        <v>0.16431676725154981</v>
+      </c>
+      <c r="F15">
+        <v>0.14730919862656239</v>
+      </c>
+      <c r="G15">
+        <v>0.14899664425751341</v>
+      </c>
+      <c r="H15">
+        <v>0.15588457268119901</v>
+      </c>
+      <c r="I15">
+        <v>8.6023252670426265E-2</v>
+      </c>
+      <c r="J15">
+        <v>0.12727922061357849</v>
+      </c>
+      <c r="K15">
+        <v>0.4476605857119878</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15" s="17">
+        <f>C15-C5</f>
+        <v>-0.42958620001005665</v>
+      </c>
+      <c r="N15" s="17">
+        <f t="shared" ref="N15:U22" si="0">D15-D5</f>
+        <v>-2.0136520692121684E-3</v>
+      </c>
+      <c r="O15" s="17">
+        <f t="shared" si="0"/>
+        <v>1.0044281046134723E-2</v>
+      </c>
+      <c r="P15" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.3100746664146084</v>
+      </c>
+      <c r="Q15" s="17">
+        <f t="shared" si="0"/>
+        <v>7.6195545364708225E-2</v>
+      </c>
+      <c r="R15" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.18086459212845571</v>
+      </c>
+      <c r="S15" s="17">
+        <f t="shared" si="0"/>
+        <v>4.2434263235019531E-2</v>
+      </c>
+      <c r="T15" s="17">
+        <f t="shared" si="0"/>
+        <v>-3.9153949157353901E-2</v>
+      </c>
+      <c r="U15" s="17">
+        <f t="shared" si="0"/>
+        <v>0.27301809374625796</v>
+      </c>
+    </row>
+    <row r="16" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C16">
+        <v>6.4031242374328487E-2</v>
+      </c>
+      <c r="D16">
+        <v>9.899494936611665E-2</v>
+      </c>
+      <c r="E16">
+        <v>0.1774823934929885</v>
+      </c>
+      <c r="F16">
+        <v>0.10049875621120891</v>
+      </c>
+      <c r="G16">
+        <v>0.1135781669160055</v>
+      </c>
+      <c r="H16">
+        <v>9.1104335791443003E-2</v>
+      </c>
+      <c r="I16">
+        <v>0.2083266665599966</v>
+      </c>
+      <c r="J16">
+        <v>0.15588457268119901</v>
+      </c>
+      <c r="K16">
+        <v>0.81326502445389848</v>
+      </c>
+      <c r="L16">
+        <v>2</v>
+      </c>
+      <c r="M16" s="17">
+        <f t="shared" ref="M16:M22" si="1">C16-C6</f>
+        <v>-3.0308568946237555E-2</v>
+      </c>
+      <c r="N16" s="17">
+        <f t="shared" si="0"/>
+        <v>-5.4302147801442255E-2</v>
+      </c>
+      <c r="O16" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.14840102124301802</v>
+      </c>
+      <c r="P16" s="17">
+        <f t="shared" si="0"/>
+        <v>2.1758677471090795E-2</v>
+      </c>
+      <c r="Q16" s="17">
+        <f t="shared" si="0"/>
+        <v>2.1926653016888689E-2</v>
+      </c>
+      <c r="R16" s="17">
+        <f t="shared" si="0"/>
+        <v>-5.0670132996135292E-2</v>
+      </c>
+      <c r="S16" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.16396354281972908</v>
+      </c>
+      <c r="T16" s="17">
+        <f t="shared" si="0"/>
+        <v>0.13352389290620112</v>
+      </c>
+      <c r="U16" s="17">
+        <f t="shared" si="0"/>
+        <v>5.9739975102518272E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C17">
+        <v>9.6953597148326576E-2</v>
+      </c>
+      <c r="D17">
+        <v>0.1367479433117734</v>
+      </c>
+      <c r="E17">
+        <v>4.2426406871192847E-2</v>
+      </c>
+      <c r="F17">
+        <v>0.43011626335213132</v>
+      </c>
+      <c r="G17">
+        <v>3.1622776601683791E-2</v>
+      </c>
+      <c r="H17">
+        <v>0.19748417658131501</v>
+      </c>
+      <c r="I17">
+        <v>0.03</v>
+      </c>
+      <c r="J17">
+        <v>0.05</v>
+      </c>
+      <c r="K17">
+        <v>0.02</v>
+      </c>
+      <c r="L17">
+        <v>3</v>
+      </c>
+      <c r="M17" s="17">
+        <f t="shared" si="1"/>
+        <v>-0.23979556766132815</v>
+      </c>
+      <c r="N17" s="17">
+        <f t="shared" si="0"/>
+        <v>-3.6168221346132512E-2</v>
+      </c>
+      <c r="O17" s="17">
+        <f t="shared" si="0"/>
+        <v>-7.9639149286144156E-2</v>
+      </c>
+      <c r="P17" s="17">
+        <f t="shared" si="0"/>
+        <v>5.4217340767881206E-2</v>
+      </c>
+      <c r="Q17" s="17">
+        <f t="shared" si="0"/>
+        <v>-4.0488248907595989E-2</v>
+      </c>
+      <c r="R17" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.23111820325342181</v>
+      </c>
+      <c r="S17" s="17">
+        <f t="shared" si="0"/>
+        <v>1.585786437626905E-2</v>
+      </c>
+      <c r="T17" s="17">
+        <f t="shared" si="0"/>
+        <v>-9.9019513592784464E-4</v>
+      </c>
+      <c r="U17" s="17">
+        <f t="shared" si="0"/>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="18" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C18">
+        <v>0.36262928728937488</v>
+      </c>
+      <c r="D18">
+        <v>8.7177978870813466E-2</v>
+      </c>
+      <c r="E18">
+        <v>0.2004993765576342</v>
+      </c>
+      <c r="F18">
+        <v>0.16792855623746669</v>
+      </c>
+      <c r="G18">
+        <v>0.12688577540449519</v>
+      </c>
+      <c r="H18">
+        <v>0.26400757564888172</v>
+      </c>
+      <c r="I18">
+        <v>5.9160797830996162E-2</v>
+      </c>
+      <c r="J18">
+        <v>0.10677078252031311</v>
+      </c>
+      <c r="K18">
+        <v>4.123105625617661E-2</v>
+      </c>
+      <c r="L18">
+        <v>4</v>
+      </c>
+      <c r="M18" s="17">
+        <f t="shared" si="1"/>
+        <v>0.24056373113203788</v>
+      </c>
+      <c r="N18" s="17">
+        <f t="shared" si="0"/>
+        <v>-9.3929723891934824E-2</v>
+      </c>
+      <c r="O18" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.11159035412891052</v>
+      </c>
+      <c r="P18" s="17">
+        <f t="shared" si="0"/>
+        <v>-1.4554319671479909E-2</v>
+      </c>
+      <c r="Q18" s="17">
+        <f t="shared" si="0"/>
+        <v>7.7895980548831636E-2</v>
+      </c>
+      <c r="R18" s="17">
+        <f t="shared" si="0"/>
+        <v>-8.3267531434825071E-2</v>
+      </c>
+      <c r="S18" s="17">
+        <f t="shared" si="0"/>
+        <v>2.3105285076356272E-2</v>
+      </c>
+      <c r="T18" s="17">
+        <f t="shared" si="0"/>
+        <v>8.9450274444624334E-2</v>
+      </c>
+      <c r="U18" s="17">
+        <f t="shared" si="0"/>
+        <v>-6.8768943743823391E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C19">
+        <v>4.2426406871192847E-2</v>
+      </c>
+      <c r="D19">
+        <v>0.21840329667841549</v>
+      </c>
+      <c r="E19">
+        <v>1.4142135623730951E-2</v>
+      </c>
+      <c r="F19">
+        <v>0.38183766184073559</v>
+      </c>
+      <c r="G19">
+        <v>0.21307275752662519</v>
+      </c>
+      <c r="H19">
+        <v>0.2437211521390788</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>0.01</v>
+      </c>
+      <c r="K19">
+        <v>2.2360679774997901E-2</v>
+      </c>
+      <c r="L19">
+        <v>5</v>
+      </c>
+      <c r="M19" s="17">
+        <f t="shared" si="1"/>
+        <v>-9.8286065923510052E-2</v>
+      </c>
+      <c r="N19" s="17">
+        <f t="shared" si="0"/>
+        <v>4.5487132020509691E-2</v>
+      </c>
+      <c r="O19" s="17">
+        <f t="shared" si="0"/>
+        <v>1.4142135623730951E-2</v>
+      </c>
+      <c r="P19" s="17">
+        <f t="shared" si="0"/>
+        <v>-9.697777168302335E-3</v>
+      </c>
+      <c r="Q19" s="17">
+        <f t="shared" si="0"/>
+        <v>3.8430265560895377E-2</v>
+      </c>
+      <c r="R19" s="17">
+        <f t="shared" si="0"/>
+        <v>-9.7013348608937622E-2</v>
+      </c>
+      <c r="S19" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="T19" s="17">
+        <f t="shared" si="0"/>
+        <v>0.01</v>
+      </c>
+      <c r="U19" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C20">
+        <v>5.385164807134505E-2</v>
+      </c>
+      <c r="D20">
+        <v>0.21213203435596431</v>
+      </c>
+      <c r="E20">
+        <v>3.7416573867739417E-2</v>
+      </c>
+      <c r="F20">
+        <v>4.123105625617661E-2</v>
+      </c>
+      <c r="G20">
+        <v>0.24124676163629641</v>
+      </c>
+      <c r="H20">
+        <v>4.123105625617661E-2</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>1.4142135623730951E-2</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>6</v>
+      </c>
+      <c r="M20" s="17">
+        <f t="shared" si="1"/>
+        <v>2.8614529354172025E-3</v>
+      </c>
+      <c r="N20" s="17">
+        <f t="shared" si="0"/>
+        <v>4.4501488213562201E-2</v>
+      </c>
+      <c r="O20" s="17">
+        <f t="shared" si="0"/>
+        <v>2.3274438244008468E-2</v>
+      </c>
+      <c r="P20" s="17">
+        <f t="shared" si="0"/>
+        <v>-3.8768943743823392E-2</v>
+      </c>
+      <c r="Q20" s="17">
+        <f t="shared" si="0"/>
+        <v>-2.063739575632384E-3</v>
+      </c>
+      <c r="R20" s="17">
+        <f t="shared" si="0"/>
+        <v>-6.1238451403419394E-2</v>
+      </c>
+      <c r="S20" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="T20" s="17">
+        <f t="shared" si="0"/>
+        <v>-1.7480640977952842E-2</v>
+      </c>
+      <c r="U20" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C21">
+        <v>7.2801098892805186E-2</v>
+      </c>
+      <c r="D21">
+        <v>0.216794833886788</v>
+      </c>
+      <c r="E21">
+        <v>2.2360679774997901E-2</v>
+      </c>
+      <c r="F21">
+        <v>8.2462112512353219E-2</v>
+      </c>
+      <c r="G21">
+        <v>0.29120439557122069</v>
+      </c>
+      <c r="H21">
+        <v>0.13190905958272919</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <v>7</v>
+      </c>
+      <c r="M21" s="17">
+        <f t="shared" si="1"/>
+        <v>6.2801098892805191E-2</v>
+      </c>
+      <c r="N21" s="17">
+        <f t="shared" si="0"/>
+        <v>2.3404037828650803E-2</v>
+      </c>
+      <c r="O21" s="17">
+        <f t="shared" si="0"/>
+        <v>2.2360679774997901E-2</v>
+      </c>
+      <c r="P21" s="17">
+        <f t="shared" si="0"/>
+        <v>8.2462112512353219E-2</v>
+      </c>
+      <c r="Q21" s="17">
+        <f t="shared" si="0"/>
+        <v>1.8257514292097099E-2</v>
+      </c>
+      <c r="R21" s="17">
+        <f t="shared" si="0"/>
+        <v>0.1219090595827292</v>
+      </c>
+      <c r="S21" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="T21" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.01</v>
+      </c>
+      <c r="U21" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="C22">
+        <v>0.92493242996448122</v>
+      </c>
+      <c r="D22">
+        <v>1.089082182390291</v>
+      </c>
+      <c r="E22">
+        <v>0.32155870381627061</v>
+      </c>
+      <c r="F22">
+        <v>1.5417198189035519</v>
+      </c>
+      <c r="G22">
+        <v>1.1636580253665589</v>
+      </c>
+      <c r="H22">
+        <v>1.872404870747777</v>
+      </c>
+      <c r="I22">
+        <v>0.29748949561287041</v>
+      </c>
+      <c r="J22">
+        <v>1.0658799181896621</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="L22">
+        <v>8</v>
+      </c>
+      <c r="M22" s="17">
+        <f t="shared" si="1"/>
+        <v>-2.8947665110516816</v>
+      </c>
+      <c r="N22" s="17">
+        <f t="shared" si="0"/>
+        <v>0.12840533766049333</v>
+      </c>
+      <c r="O22" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.1086737914697084</v>
+      </c>
+      <c r="P22" s="17">
+        <f t="shared" si="0"/>
+        <v>0.46056303101384</v>
+      </c>
+      <c r="Q22" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.52563176623226604</v>
+      </c>
+      <c r="R22" s="17">
+        <f t="shared" si="0"/>
+        <v>0.360650922514137</v>
+      </c>
+      <c r="S22" s="17">
+        <f t="shared" si="0"/>
+        <v>6.1269259392516123E-2</v>
+      </c>
+      <c r="T22" s="17">
+        <f t="shared" si="0"/>
+        <v>-9.1833345101382857E-2</v>
+      </c>
+      <c r="U22" s="17">
+        <f t="shared" si="0"/>
+        <v>-0.41484937025383078</v>
       </c>
     </row>
   </sheetData>
@@ -6200,10 +7997,22 @@
     <mergeCell ref="B2:K2"/>
   </mergeCells>
   <conditionalFormatting sqref="C5:K12">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M15:U22">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FFF8696B"/>
       </colorScale>

</xml_diff>